<commit_message>
Deploying to gh-pages from  @ ff959e874c4afa79b209c58462ab7f7c0eb64507 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/1.1.1.1.xlsx
+++ b/en/downloads/data-excel/1.1.1.1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\korozbaeva\Desktop\Показатели ЦУР для Платформы\Национальные показатели ЦУР\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Показатели ЦУР для Платформы\Национальные показатели ЦУР — 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B79F9DC-19A7-417F-AC23-E8EAE7F81A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12510" windowHeight="9435"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист 1" sheetId="1" r:id="rId1"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="64">
   <si>
     <t>Көрсөткүчтөрдүн аталышы</t>
   </si>
@@ -37,9 +38,6 @@
   </si>
   <si>
     <t>Items</t>
-  </si>
-  <si>
-    <t>1.1.1.1a Уровень крайней бедности</t>
   </si>
   <si>
     <t>(в процентах к общей численности населения)</t>
@@ -75,13 +73,7 @@
     <t>Kyrgyz Republic</t>
   </si>
   <si>
-    <t xml:space="preserve">1.1.1.1a Level of extreme poverty </t>
-  </si>
-  <si>
     <t>(in percent to total population)</t>
-  </si>
-  <si>
-    <t>1.1.1.1а Деңгээли өтө жакырчылык калк</t>
   </si>
   <si>
     <t>Кыргыз Республикасы</t>
@@ -221,15 +213,26 @@
   <si>
     <t>By territory</t>
   </si>
+  <si>
+    <t xml:space="preserve">1.1.1.1 Level of extreme poverty </t>
+  </si>
+  <si>
+    <t>1.1.1.1 Уровень крайней бедности</t>
+  </si>
+  <si>
+    <t>1.1.1.1 Деңгээли өтө жакырчылык калк</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.00\ _₽_-;\-* #,##0.00\ _₽_-;_-* &quot;-&quot;??\ _₽_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="General_)"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="40">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,16 +359,268 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Courier"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman CYR"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="62"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="63"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="20"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color indexed="23"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="17"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="52"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color indexed="56"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color indexed="56"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="56"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color indexed="56"/>
+      <name val="Cambria"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="60"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Helv"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="52"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="44"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="29"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="45"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="26"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="46"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="27"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="51"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="30"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="53"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="49"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="62"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="22"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="55"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -415,8 +670,115 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="23"/>
+      </left>
+      <right style="thin">
+        <color indexed="23"/>
+      </right>
+      <top style="thin">
+        <color indexed="23"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="23"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="63"/>
+      </left>
+      <right style="thin">
+        <color indexed="63"/>
+      </right>
+      <top style="thin">
+        <color indexed="63"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="63"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="62"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="22"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="30"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="62"/>
+      </top>
+      <bottom style="double">
+        <color indexed="62"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="63"/>
+      </left>
+      <right style="double">
+        <color indexed="63"/>
+      </right>
+      <top style="double">
+        <color indexed="63"/>
+      </top>
+      <bottom style="double">
+        <color indexed="63"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="22"/>
+      </left>
+      <right style="thin">
+        <color indexed="22"/>
+      </right>
+      <top style="thin">
+        <color indexed="22"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="22"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color indexed="52"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="12">
+  <cellStyleXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -431,8 +793,56 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyFont="0" applyAlignment="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="170" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -446,20 +856,17 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -470,10 +877,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -485,45 +892,93 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="12">
-    <cellStyle name="Normal 17" xfId="3"/>
+  <cellStyles count="60">
+    <cellStyle name="20% - Акцент1 2" xfId="12" xr:uid="{251193FB-8682-4C1E-8E0A-2F8F1FFABE20}"/>
+    <cellStyle name="20% - Акцент2 2" xfId="13" xr:uid="{EB968BC2-8924-4092-B83B-859079E256E2}"/>
+    <cellStyle name="20% - Акцент3 2" xfId="14" xr:uid="{9FA8EB59-ABCE-45D3-98DE-E0F298A38816}"/>
+    <cellStyle name="20% - Акцент4 2" xfId="15" xr:uid="{72AD7ECB-752E-48CA-BD39-52F926AA557E}"/>
+    <cellStyle name="20% - Акцент5 2" xfId="16" xr:uid="{4A713BAB-384F-4641-93C8-7B7BFD546830}"/>
+    <cellStyle name="20% - Акцент6 2" xfId="17" xr:uid="{900E81E1-9EEE-4A4D-8FB7-F87386F0473E}"/>
+    <cellStyle name="40% - Акцент1 2" xfId="18" xr:uid="{74D5094F-2579-48DE-B598-F9D862A5AE2A}"/>
+    <cellStyle name="40% - Акцент2 2" xfId="19" xr:uid="{C5EC8B07-DB97-4A78-A7F7-ACCE2BA9825E}"/>
+    <cellStyle name="40% - Акцент3 2" xfId="20" xr:uid="{33D5CA21-F189-4A66-B094-97BE82F86266}"/>
+    <cellStyle name="40% - Акцент4 2" xfId="21" xr:uid="{D0AB2749-2DAD-493E-BCAF-EE342FB6338A}"/>
+    <cellStyle name="40% - Акцент5 2" xfId="22" xr:uid="{4D898A94-3542-4052-B998-B936C89DF1A1}"/>
+    <cellStyle name="40% - Акцент6 2" xfId="23" xr:uid="{0A9FF476-E899-4E43-B571-4DD623795F48}"/>
+    <cellStyle name="60% - Акцент1 2" xfId="24" xr:uid="{23EA3D95-CA50-40E1-B017-97F7F85472B5}"/>
+    <cellStyle name="60% - Акцент2 2" xfId="25" xr:uid="{6C20E318-A2C1-4ADE-9C66-795A6830CFEC}"/>
+    <cellStyle name="60% - Акцент3 2" xfId="26" xr:uid="{E45B392F-6A7D-42FB-B429-BFFA09762374}"/>
+    <cellStyle name="60% - Акцент4 2" xfId="27" xr:uid="{DBB3D191-B7D3-4DD2-B0D9-8308547B1700}"/>
+    <cellStyle name="60% - Акцент5 2" xfId="28" xr:uid="{A1132113-215C-4900-BFC1-B174B43058F0}"/>
+    <cellStyle name="60% - Акцент6 2" xfId="29" xr:uid="{C857ED8A-1A6F-4091-AFAF-0C9D4D5DC04C}"/>
+    <cellStyle name="Iau?iue_B-119603" xfId="30" xr:uid="{61713699-FEE2-4DEC-9DF9-B0DCF77B3AC2}"/>
+    <cellStyle name="Normal 17" xfId="3" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Акцент1 2" xfId="31" xr:uid="{62808C21-FBDB-4B0C-85F9-881881AB3D6B}"/>
+    <cellStyle name="Акцент2 2" xfId="32" xr:uid="{8F22370B-7E1D-439B-BDFD-BE00F3D3BC2E}"/>
+    <cellStyle name="Акцент3 2" xfId="33" xr:uid="{FBF2CD10-5033-4171-9CC6-E5344DED5A03}"/>
+    <cellStyle name="Акцент4 2" xfId="34" xr:uid="{EA2D9B98-A7E0-41AC-BC3E-6F4A18B8E3A9}"/>
+    <cellStyle name="Акцент5 2" xfId="35" xr:uid="{BB06BC0B-1DC9-4CA9-8CAD-3B899FEA2786}"/>
+    <cellStyle name="Акцент6 2" xfId="36" xr:uid="{721C91B2-C73C-4747-924C-3F1B39FB0BEB}"/>
+    <cellStyle name="Ввод  2" xfId="37" xr:uid="{DDF299C1-621E-4369-BEBB-B2DE78E0872C}"/>
+    <cellStyle name="Вывод 2" xfId="38" xr:uid="{1B7A46E5-7A68-481A-B1B4-127ED550FE26}"/>
+    <cellStyle name="Вычисление 2" xfId="39" xr:uid="{2EA539F8-604F-46A6-ADE8-4EB3004C1910}"/>
+    <cellStyle name="Заголовок 1 2" xfId="40" xr:uid="{0A0BE7FE-0165-4DF0-8558-64215503F2E3}"/>
+    <cellStyle name="Заголовок 2 2" xfId="41" xr:uid="{94F1036F-3E31-4A87-BDBD-CB597979AF77}"/>
+    <cellStyle name="Заголовок 3 2" xfId="42" xr:uid="{76F69A51-E02E-413A-A8EB-729C93C92F8D}"/>
+    <cellStyle name="Заголовок 4 2" xfId="43" xr:uid="{990863EA-6EED-42B7-AAFE-7CE48DF58134}"/>
+    <cellStyle name="Итог 2" xfId="44" xr:uid="{59ED9419-9C37-4565-8F6B-06CB6C7647AD}"/>
+    <cellStyle name="Контрольная ячейка 2" xfId="45" xr:uid="{73AC6107-6C17-42AB-92B6-9761600C420F}"/>
+    <cellStyle name="Название 2" xfId="46" xr:uid="{E0D58004-87E8-4F54-BA29-CEB901D06FE6}"/>
+    <cellStyle name="Нейтральный 2" xfId="47" xr:uid="{B40E6F5C-BE06-416B-A9DD-4933843FB40D}"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Обычный 2" xfId="1"/>
-    <cellStyle name="Обычный 2 2" xfId="10"/>
-    <cellStyle name="Обычный 2 3" xfId="5"/>
-    <cellStyle name="Обычный 3" xfId="6"/>
-    <cellStyle name="Обычный 4" xfId="9"/>
-    <cellStyle name="Обычный 6" xfId="2"/>
-    <cellStyle name="Обычный 7" xfId="4"/>
-    <cellStyle name="полужирный" xfId="11"/>
-    <cellStyle name="Процентный 2" xfId="8"/>
-    <cellStyle name="Процентный 3" xfId="7"/>
+    <cellStyle name="Обычный 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Обычный 2 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Обычный 2 2 2" xfId="49" xr:uid="{55A7A134-39EB-4554-A6C7-F88B84BA1635}"/>
+    <cellStyle name="Обычный 2 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Обычный 2 3 2" xfId="48" xr:uid="{7666E47F-45A6-4500-BB2E-21B8E4519C46}"/>
+    <cellStyle name="Обычный 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Обычный 3 2" xfId="50" xr:uid="{15E7BE22-C1C6-4E55-8CDD-3CF4B088A9C2}"/>
+    <cellStyle name="Обычный 4" xfId="9" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Обычный 5" xfId="59" xr:uid="{D12A4D71-D0E8-402A-9799-8B51DB2EBD00}"/>
+    <cellStyle name="Обычный 6" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Обычный 7" xfId="4" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Плохой 2" xfId="51" xr:uid="{9656FF66-6F0E-40A7-AC5C-3B90D5A0D106}"/>
+    <cellStyle name="полужирный" xfId="11" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Пояснение 2" xfId="52" xr:uid="{16C88423-4EB7-4263-9E8B-F8A6FC8D149E}"/>
+    <cellStyle name="Примечание 2" xfId="53" xr:uid="{986EA234-E98E-4CBA-AC23-CB057B2C5FA9}"/>
+    <cellStyle name="Процентный 2" xfId="8" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Процентный 3" xfId="7" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Связанная ячейка 2" xfId="54" xr:uid="{16BF78FF-96EB-46DB-BC20-20C12C0D0C2A}"/>
+    <cellStyle name="Стиль 1" xfId="55" xr:uid="{7642EC21-3B84-48F6-92CB-AD0C3432887C}"/>
+    <cellStyle name="Текст предупреждения 2" xfId="56" xr:uid="{3BEDEF0C-7D71-49A4-B0B8-F3BD25D538B0}"/>
+    <cellStyle name="Финансовый 2" xfId="57" xr:uid="{4037D2C5-AF23-49C4-99D4-217C0FF089CD}"/>
+    <cellStyle name="Хороший 2" xfId="58" xr:uid="{0D375FC1-4B06-4C94-A4F6-2417852BBA72}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -539,7 +994,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Data"/>
@@ -8265,54 +8720,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R22"/>
   <sheetFormatPr defaultRowHeight="12"/>
   <cols>
-    <col min="1" max="3" width="35" style="2" customWidth="1"/>
+    <col min="1" max="3" width="34.28515625" style="2" customWidth="1"/>
     <col min="4" max="7" width="11.140625" style="2" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="24" customHeight="1">
-      <c r="A1" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="17" t="s">
+    <row r="1" spans="1:18" ht="24" customHeight="1">
+      <c r="A1" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="13.5" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="17" t="s">
-        <v>15</v>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="13.5" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>16</v>
-      </c>
+    <row r="3" spans="1:18" ht="13.5" customHeight="1" thickBot="1">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="33"/>
     </row>
-    <row r="3" spans="1:17" ht="13.5" customHeight="1" thickBot="1">
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-    </row>
-    <row r="4" spans="1:17" ht="14.25" customHeight="1" thickBot="1">
+    <row r="4" spans="1:18" ht="14.25" customHeight="1" thickBot="1">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -8322,869 +8778,923 @@
       <c r="C4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="11">
         <v>2010</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="11">
         <v>2011</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="11">
         <v>2012</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="11">
         <v>2013</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="11">
         <v>2014</v>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="11">
         <v>2015</v>
       </c>
-      <c r="J4" s="12">
+      <c r="J4" s="11">
         <v>2016</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="11">
         <v>2017</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="11">
         <v>2018</v>
       </c>
-      <c r="M4" s="12">
+      <c r="M4" s="11">
         <v>2019</v>
       </c>
-      <c r="N4" s="18">
+      <c r="N4" s="17">
         <v>2020</v>
       </c>
-      <c r="O4" s="18">
+      <c r="O4" s="17">
         <v>2021</v>
       </c>
-      <c r="P4" s="18">
+      <c r="P4" s="17">
         <v>2022</v>
       </c>
-      <c r="Q4" s="18">
+      <c r="Q4" s="17">
         <v>2023</v>
       </c>
+      <c r="R4" s="29">
+        <v>2024</v>
+      </c>
     </row>
-    <row r="5" spans="1:17" ht="14.25" customHeight="1">
+    <row r="5" spans="1:18" ht="14.25" customHeight="1">
       <c r="A5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="12">
+        <v>5.3438169958924879</v>
+      </c>
+      <c r="E5" s="12">
+        <v>4.545728690156194</v>
+      </c>
+      <c r="F5" s="12">
+        <v>4.3902104224137357</v>
+      </c>
+      <c r="G5" s="12">
+        <v>2.7520531699173962</v>
+      </c>
+      <c r="H5" s="12">
+        <v>1.2045438763134317</v>
+      </c>
+      <c r="I5" s="12">
+        <v>1.2463</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0.79950533734625018</v>
+      </c>
+      <c r="K5" s="12">
+        <v>0.75126418709986076</v>
+      </c>
+      <c r="L5" s="12">
+        <v>0.55684909247351222</v>
+      </c>
+      <c r="M5" s="12">
+        <v>0.54933623931578479</v>
+      </c>
+      <c r="N5" s="18">
+        <v>0.89148765717852163</v>
+      </c>
+      <c r="O5" s="18">
+        <v>6.0337796775071091</v>
+      </c>
+      <c r="P5" s="18">
+        <v>5.9676405075953687</v>
+      </c>
+      <c r="Q5" s="18">
+        <v>4.9547183120610843</v>
+      </c>
+      <c r="R5" s="30">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" customFormat="1" ht="15">
+      <c r="A6" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
+      <c r="R6" s="31"/>
+    </row>
+    <row r="7" spans="1:18" customFormat="1" ht="15">
+      <c r="A7" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" s="26">
+        <v>0.68519413875264201</v>
+      </c>
+      <c r="L7" s="26">
+        <v>0.52778295592322599</v>
+      </c>
+      <c r="M7" s="26">
+        <v>0.55180198070156894</v>
+      </c>
+      <c r="N7" s="26">
+        <v>0.80960724343075641</v>
+      </c>
+      <c r="O7" s="26">
+        <v>6.2123810703447084</v>
+      </c>
+      <c r="P7" s="26">
+        <v>6.2</v>
+      </c>
+      <c r="Q7" s="26">
+        <v>4.9263803296199171</v>
+      </c>
+      <c r="R7" s="31">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" customFormat="1" ht="15">
+      <c r="A8" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" s="26">
+        <v>0.82404503217287961</v>
+      </c>
+      <c r="L8" s="26">
+        <v>0.589459031995476</v>
+      </c>
+      <c r="M8" s="26">
+        <v>0.54655576288689411</v>
+      </c>
+      <c r="N8" s="26">
+        <v>0.98245128998233044</v>
+      </c>
+      <c r="O8" s="26">
+        <v>5.8348173264224643</v>
+      </c>
+      <c r="P8" s="26">
+        <v>5.7</v>
+      </c>
+      <c r="Q8" s="26">
+        <v>4.9857836040976133</v>
+      </c>
+      <c r="R8" s="31">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" customFormat="1" ht="15">
+      <c r="A9" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="26"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="26"/>
+      <c r="R9" s="31"/>
+    </row>
+    <row r="10" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="13">
+        <v>4.2168631530813512</v>
+      </c>
+      <c r="E10" s="13">
+        <v>2.5713927856479444</v>
+      </c>
+      <c r="F10" s="13">
+        <v>4.2453039507137298</v>
+      </c>
+      <c r="G10" s="13">
+        <v>1.622592666205378</v>
+      </c>
+      <c r="H10" s="13">
+        <v>1.3352534216041274</v>
+      </c>
+      <c r="I10" s="13">
+        <v>1.0364</v>
+      </c>
+      <c r="J10" s="13">
+        <v>0.32993924401723507</v>
+      </c>
+      <c r="K10" s="13">
+        <v>0.31702172210916746</v>
+      </c>
+      <c r="L10" s="13">
+        <v>0.2403586586679928</v>
+      </c>
+      <c r="M10" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="N10" s="19">
+        <v>0.31407178438278893</v>
+      </c>
+      <c r="O10" s="22">
+        <v>7.3075058743442511</v>
+      </c>
+      <c r="P10" s="22">
+        <v>5.6044335798150424</v>
+      </c>
+      <c r="Q10" s="22">
+        <v>5.2409183200762754</v>
+      </c>
+      <c r="R10" s="31">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="13">
+        <v>5.9930922559799589</v>
+      </c>
+      <c r="E11" s="13">
+        <v>5.7195315396021638</v>
+      </c>
+      <c r="F11" s="13">
+        <v>4.474039629820532</v>
+      </c>
+      <c r="G11" s="13">
+        <v>3.3387697541408841</v>
+      </c>
+      <c r="H11" s="13">
+        <v>1.1307049829892899</v>
+      </c>
+      <c r="I11" s="13">
+        <v>1.3613</v>
+      </c>
+      <c r="J11" s="13">
+        <v>1.0572316812127296</v>
+      </c>
+      <c r="K11" s="13">
+        <v>0.9904939556603013</v>
+      </c>
+      <c r="L11" s="13">
+        <v>0.7328783431070176</v>
+      </c>
+      <c r="M11" s="13">
+        <v>0.8</v>
+      </c>
+      <c r="N11" s="19">
+        <v>1.220561325080239</v>
+      </c>
+      <c r="O11" s="22">
+        <v>5.2767607763499562</v>
+      </c>
+      <c r="P11" s="22">
+        <v>6.1789553077823856</v>
+      </c>
+      <c r="Q11" s="22">
+        <v>4.7888452943619573</v>
+      </c>
+      <c r="R11" s="31">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" customFormat="1" ht="15">
+      <c r="A12" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="28"/>
+      <c r="M12" s="26"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="26"/>
+      <c r="P12" s="26"/>
+      <c r="Q12" s="26"/>
+      <c r="R12" s="31"/>
+    </row>
+    <row r="13" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="13">
-        <v>5.3438169958924879</v>
-      </c>
-      <c r="E5" s="13">
-        <v>4.545728690156194</v>
-      </c>
-      <c r="F5" s="13">
-        <v>4.3902104224137357</v>
-      </c>
-      <c r="G5" s="13">
-        <v>2.7520531699173962</v>
-      </c>
-      <c r="H5" s="13">
-        <v>1.2045438763134317</v>
-      </c>
-      <c r="I5" s="13">
-        <v>1.2463</v>
-      </c>
-      <c r="J5" s="13">
-        <v>0.79950533734625018</v>
-      </c>
-      <c r="K5" s="13">
-        <v>0.75126418709986076</v>
-      </c>
-      <c r="L5" s="13">
-        <v>0.55684909247351222</v>
-      </c>
-      <c r="M5" s="13">
-        <v>0.54933623931578479</v>
-      </c>
-      <c r="N5" s="19">
-        <v>0.89148765717852163</v>
-      </c>
-      <c r="O5" s="19">
-        <v>6.0337796775071091</v>
-      </c>
-      <c r="P5" s="19">
-        <v>5.9676405075953687</v>
-      </c>
-      <c r="Q5" s="19">
-        <v>4.9547183120610843</v>
+      <c r="D13" s="13">
+        <v>5.1808804816231708</v>
+      </c>
+      <c r="E13" s="13">
+        <v>3.5712525519800784</v>
+      </c>
+      <c r="F13" s="13">
+        <v>2.4298219022359215</v>
+      </c>
+      <c r="G13" s="13">
+        <v>7.9920581957878776</v>
+      </c>
+      <c r="H13" s="13">
+        <v>2.6473978814209165</v>
+      </c>
+      <c r="I13" s="13">
+        <v>4.0069999999999997</v>
+      </c>
+      <c r="J13" s="13">
+        <v>0.32112435111554388</v>
+      </c>
+      <c r="K13" s="13">
+        <v>3.3941360063781501</v>
+      </c>
+      <c r="L13" s="13">
+        <v>0.87300583877555049</v>
+      </c>
+      <c r="M13" s="13">
+        <v>0.3392671909690585</v>
+      </c>
+      <c r="N13" s="20">
+        <v>1.6290305205827647</v>
+      </c>
+      <c r="O13" s="22">
+        <v>10.064200140319592</v>
+      </c>
+      <c r="P13" s="22">
+        <v>16.5</v>
+      </c>
+      <c r="Q13" s="22">
+        <v>16.145310230913825</v>
+      </c>
+      <c r="R13" s="31">
+        <v>11.8</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="28" customFormat="1" ht="15">
-      <c r="A6" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="26" t="s">
+    <row r="14" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="13">
+        <v>6.4380322738993074</v>
+      </c>
+      <c r="E14" s="13">
+        <v>6.6554187654394825</v>
+      </c>
+      <c r="F14" s="13">
+        <v>14.126082809346473</v>
+      </c>
+      <c r="G14" s="13">
+        <v>1.4181571804450666</v>
+      </c>
+      <c r="H14" s="13">
+        <v>1.06205582454581</v>
+      </c>
+      <c r="I14" s="13">
+        <v>0.47739999999999999</v>
+      </c>
+      <c r="J14" s="13">
+        <v>0.11107551172966013</v>
+      </c>
+      <c r="K14" s="13">
+        <v>0</v>
+      </c>
+      <c r="L14" s="13">
+        <v>1.011691375024679</v>
+      </c>
+      <c r="M14" s="13">
+        <v>0.56205045247263075</v>
+      </c>
+      <c r="N14" s="20">
+        <v>1.4841131607226035</v>
+      </c>
+      <c r="O14" s="22">
+        <v>7.5445007460298559</v>
+      </c>
+      <c r="P14" s="22">
+        <v>9.1</v>
+      </c>
+      <c r="Q14" s="22">
+        <v>5.0414052649559933</v>
+      </c>
+      <c r="R14" s="31">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="13">
+        <v>2.4787267316625954</v>
+      </c>
+      <c r="E15" s="13">
+        <v>1.5072935699864518</v>
+      </c>
+      <c r="F15" s="13">
+        <v>0.13114731930321041</v>
+      </c>
+      <c r="G15" s="13">
+        <v>1.9058703261018888</v>
+      </c>
+      <c r="H15" s="13">
+        <v>0</v>
+      </c>
+      <c r="I15" s="13">
+        <v>0.41110000000000002</v>
+      </c>
+      <c r="J15" s="13">
+        <v>0</v>
+      </c>
+      <c r="K15" s="13">
+        <v>1.0368879452299757</v>
+      </c>
+      <c r="L15" s="13">
+        <v>0.89229699812925367</v>
+      </c>
+      <c r="M15" s="13">
+        <v>1.2604968981368243</v>
+      </c>
+      <c r="N15" s="20">
+        <v>0.43494800834006392</v>
+      </c>
+      <c r="O15" s="22">
+        <v>7.9562092224762884</v>
+      </c>
+      <c r="P15" s="22">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="Q15" s="22">
+        <v>7.2304756924160642</v>
+      </c>
+      <c r="R15" s="31">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="13">
+        <v>12.036462028653192</v>
+      </c>
+      <c r="E16" s="13">
+        <v>14.690826870034272</v>
+      </c>
+      <c r="F16" s="13">
+        <v>2.4571173079700253</v>
+      </c>
+      <c r="G16" s="13">
+        <v>4.8604171260649736</v>
+      </c>
+      <c r="H16" s="13">
+        <v>1.8174089333614543</v>
+      </c>
+      <c r="I16" s="13">
+        <v>2.0588000000000002</v>
+      </c>
+      <c r="J16" s="13">
+        <v>2.566584561254897</v>
+      </c>
+      <c r="K16" s="13">
+        <v>1.9537658797263695</v>
+      </c>
+      <c r="L16" s="13">
+        <v>2.1781909222789975</v>
+      </c>
+      <c r="M16" s="13">
+        <v>2.4816289901846873</v>
+      </c>
+      <c r="N16" s="20">
+        <v>4.5037215639801795</v>
+      </c>
+      <c r="O16" s="22">
+        <v>8.1696953402867685</v>
+      </c>
+      <c r="P16" s="22">
+        <v>6.7</v>
+      </c>
+      <c r="Q16" s="22">
+        <v>5.636136560567035</v>
+      </c>
+      <c r="R16" s="31">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="13">
+        <v>8.3331494569001308</v>
+      </c>
+      <c r="E17" s="13">
+        <v>3.6874208696079878</v>
+      </c>
+      <c r="F17" s="13">
+        <v>2.2967063175794622</v>
+      </c>
+      <c r="G17" s="13">
+        <v>4.0113695837012733</v>
+      </c>
+      <c r="H17" s="13">
+        <v>0.42340246664306652</v>
+      </c>
+      <c r="I17" s="13">
+        <v>1.1879</v>
+      </c>
+      <c r="J17" s="13">
+        <v>0.82824784717641098</v>
+      </c>
+      <c r="K17" s="13">
+        <v>0</v>
+      </c>
+      <c r="L17" s="13">
+        <v>0</v>
+      </c>
+      <c r="M17" s="13">
+        <v>0.88079865305212723</v>
+      </c>
+      <c r="N17" s="20">
+        <v>0</v>
+      </c>
+      <c r="O17" s="22">
+        <v>2.0701729813092102</v>
+      </c>
+      <c r="P17" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="Q17" s="22">
+        <v>0.28220429532766028</v>
+      </c>
+      <c r="R17" s="31">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="13">
+        <v>5.0122940777216947</v>
+      </c>
+      <c r="E18" s="13">
+        <v>8.4390180594440558</v>
+      </c>
+      <c r="F18" s="13">
+        <v>0.9048113995307433</v>
+      </c>
+      <c r="G18" s="13">
+        <v>0</v>
+      </c>
+      <c r="H18" s="13">
+        <v>0</v>
+      </c>
+      <c r="I18" s="13">
+        <v>0</v>
+      </c>
+      <c r="J18" s="13">
+        <v>0</v>
+      </c>
+      <c r="K18" s="13">
+        <v>0</v>
+      </c>
+      <c r="L18" s="13">
+        <v>0</v>
+      </c>
+      <c r="M18" s="13">
+        <v>0</v>
+      </c>
+      <c r="N18" s="20">
+        <v>0</v>
+      </c>
+      <c r="O18" s="22">
+        <v>2.6482523478927704</v>
+      </c>
+      <c r="P18" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="Q18" s="22">
+        <v>4.1787877227366739</v>
+      </c>
+      <c r="R18" s="31">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="13">
+        <v>3.5353129806100583</v>
+      </c>
+      <c r="E19" s="13">
+        <v>4.8599509512033325</v>
+      </c>
+      <c r="F19" s="13">
+        <v>3.8945633266892905</v>
+      </c>
+      <c r="G19" s="13">
+        <v>2.0810969960991046</v>
+      </c>
+      <c r="H19" s="13">
+        <v>3.1927887343841532</v>
+      </c>
+      <c r="I19" s="13">
+        <v>1.6887000000000001</v>
+      </c>
+      <c r="J19" s="13">
+        <v>3.1263372864926211</v>
+      </c>
+      <c r="K19" s="13">
+        <v>1.6870705087645406</v>
+      </c>
+      <c r="L19" s="13">
+        <v>0.32414908639895251</v>
+      </c>
+      <c r="M19" s="13">
+        <v>0.16260204281171109</v>
+      </c>
+      <c r="N19" s="20">
+        <v>1.3481169038547842</v>
+      </c>
+      <c r="O19" s="22">
+        <v>3.9561647100749857</v>
+      </c>
+      <c r="P19" s="22">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="Q19" s="22">
+        <v>4.5216072733589767</v>
+      </c>
+      <c r="R19" s="31">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="14.25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="13">
+        <v>0.53092532677015958</v>
+      </c>
+      <c r="E20" s="13">
+        <v>1.0193281509036862</v>
+      </c>
+      <c r="F20" s="13">
+        <v>1.1684706283465978</v>
+      </c>
+      <c r="G20" s="13">
+        <v>0.96005330035931602</v>
+      </c>
+      <c r="H20" s="13">
+        <v>0</v>
+      </c>
+      <c r="I20" s="13">
+        <v>0.78439999999999999</v>
+      </c>
+      <c r="J20" s="13">
+        <v>0</v>
+      </c>
+      <c r="K20" s="13">
+        <v>0</v>
+      </c>
+      <c r="L20" s="13">
+        <v>0.32812063618010201</v>
+      </c>
+      <c r="M20" s="13">
+        <v>0</v>
+      </c>
+      <c r="N20" s="20">
+        <v>0.28229127286371936</v>
+      </c>
+      <c r="O20" s="22">
+        <v>9.4645167179465837</v>
+      </c>
+      <c r="P20" s="22">
+        <v>3.9</v>
+      </c>
+      <c r="Q20" s="22">
+        <v>5.6913920534882436</v>
+      </c>
+      <c r="R20" s="31">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="14.25" customHeight="1" thickBot="1">
+      <c r="A21" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
+      <c r="E21" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="15">
+        <v>3.5070632421313164</v>
+      </c>
+      <c r="H21" s="15">
+        <v>3.1020289567965551</v>
+      </c>
+      <c r="I21" s="15">
+        <v>1.7009000000000001</v>
+      </c>
+      <c r="J21" s="15">
+        <v>0</v>
+      </c>
+      <c r="K21" s="15">
+        <v>1.1812990540391501</v>
+      </c>
+      <c r="L21" s="15">
+        <v>0.55610781362635098</v>
+      </c>
+      <c r="M21" s="15">
+        <v>0</v>
+      </c>
+      <c r="N21" s="21">
+        <v>0</v>
+      </c>
+      <c r="O21" s="23">
+        <v>3.1019579996103404</v>
+      </c>
+      <c r="P21" s="23">
+        <v>7</v>
+      </c>
+      <c r="Q21" s="23">
+        <v>1.3988584602956362</v>
+      </c>
+      <c r="R21" s="32">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:17" s="28" customFormat="1" ht="15">
-      <c r="A7" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="I7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" s="27">
-        <v>0.68519413875264201</v>
-      </c>
-      <c r="L7" s="27">
-        <v>0.52778295592322599</v>
-      </c>
-      <c r="M7" s="27">
-        <v>0.55180198070156894</v>
-      </c>
-      <c r="N7" s="27">
-        <v>0.80960724343075641</v>
-      </c>
-      <c r="O7" s="27">
-        <v>6.2123810703447084</v>
-      </c>
-      <c r="P7" s="27">
-        <v>6.2</v>
-      </c>
-      <c r="Q7" s="27">
-        <v>4.9263803296199171</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" s="28" customFormat="1" ht="15">
-      <c r="A8" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="H8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="J8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="27">
-        <v>0.82404503217287961</v>
-      </c>
-      <c r="L8" s="27">
-        <v>0.589459031995476</v>
-      </c>
-      <c r="M8" s="27">
-        <v>0.54655576288689411</v>
-      </c>
-      <c r="N8" s="27">
-        <v>0.98245128998233044</v>
-      </c>
-      <c r="O8" s="27">
-        <v>5.8348173264224643</v>
-      </c>
-      <c r="P8" s="27">
-        <v>5.7</v>
-      </c>
-      <c r="Q8" s="27">
-        <v>4.9857836040976133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" s="28" customFormat="1" ht="15">
-      <c r="A9" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="27"/>
-    </row>
-    <row r="10" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A10" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="14">
-        <v>4.2168631530813512</v>
-      </c>
-      <c r="E10" s="14">
-        <v>2.5713927856479444</v>
-      </c>
-      <c r="F10" s="14">
-        <v>4.2453039507137298</v>
-      </c>
-      <c r="G10" s="14">
-        <v>1.622592666205378</v>
-      </c>
-      <c r="H10" s="14">
-        <v>1.3352534216041274</v>
-      </c>
-      <c r="I10" s="14">
-        <v>1.0364</v>
-      </c>
-      <c r="J10" s="14">
-        <v>0.32993924401723507</v>
-      </c>
-      <c r="K10" s="14">
-        <v>0.31702172210916746</v>
-      </c>
-      <c r="L10" s="14">
-        <v>0.2403586586679928</v>
-      </c>
-      <c r="M10" s="14">
-        <v>0.1</v>
-      </c>
-      <c r="N10" s="20">
-        <v>0.31407178438278893</v>
-      </c>
-      <c r="O10" s="23">
-        <v>7.3075058743442511</v>
-      </c>
-      <c r="P10" s="23">
-        <v>5.6044335798150424</v>
-      </c>
-      <c r="Q10" s="23">
-        <v>5.2409183200762754</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="14">
-        <v>5.9930922559799589</v>
-      </c>
-      <c r="E11" s="14">
-        <v>5.7195315396021638</v>
-      </c>
-      <c r="F11" s="14">
-        <v>4.474039629820532</v>
-      </c>
-      <c r="G11" s="14">
-        <v>3.3387697541408841</v>
-      </c>
-      <c r="H11" s="14">
-        <v>1.1307049829892899</v>
-      </c>
-      <c r="I11" s="14">
-        <v>1.3613</v>
-      </c>
-      <c r="J11" s="14">
-        <v>1.0572316812127296</v>
-      </c>
-      <c r="K11" s="14">
-        <v>0.9904939556603013</v>
-      </c>
-      <c r="L11" s="14">
-        <v>0.7328783431070176</v>
-      </c>
-      <c r="M11" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="N11" s="20">
-        <v>1.220561325080239</v>
-      </c>
-      <c r="O11" s="23">
-        <v>5.2767607763499562</v>
-      </c>
-      <c r="P11" s="23">
-        <v>6.1789553077823856</v>
-      </c>
-      <c r="Q11" s="23">
-        <v>4.7888452943619573</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" customFormat="1" ht="15">
-      <c r="A12" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="31" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
-      <c r="K12" s="27"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="27"/>
-      <c r="N12" s="27"/>
-      <c r="O12" s="27"/>
-      <c r="P12" s="27"/>
-      <c r="Q12" s="27"/>
-    </row>
-    <row r="13" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="14">
-        <v>5.1808804816231708</v>
-      </c>
-      <c r="E13" s="14">
-        <v>3.5712525519800784</v>
-      </c>
-      <c r="F13" s="14">
-        <v>2.4298219022359215</v>
-      </c>
-      <c r="G13" s="14">
-        <v>7.9920581957878776</v>
-      </c>
-      <c r="H13" s="14">
-        <v>2.6473978814209165</v>
-      </c>
-      <c r="I13" s="14">
-        <v>4.0069999999999997</v>
-      </c>
-      <c r="J13" s="14">
-        <v>0.32112435111554388</v>
-      </c>
-      <c r="K13" s="14">
-        <v>3.3941360063781501</v>
-      </c>
-      <c r="L13" s="14">
-        <v>0.87300583877555049</v>
-      </c>
-      <c r="M13" s="14">
-        <v>0.3392671909690585</v>
-      </c>
-      <c r="N13" s="21">
-        <v>1.6290305205827647</v>
-      </c>
-      <c r="O13" s="23">
-        <v>10.064200140319592</v>
-      </c>
-      <c r="P13" s="23">
-        <v>16.5</v>
-      </c>
-      <c r="Q13" s="23">
-        <v>16.145310230913825</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="14">
-        <v>6.4380322738993074</v>
-      </c>
-      <c r="E14" s="14">
-        <v>6.6554187654394825</v>
-      </c>
-      <c r="F14" s="14">
-        <v>14.126082809346473</v>
-      </c>
-      <c r="G14" s="14">
-        <v>1.4181571804450666</v>
-      </c>
-      <c r="H14" s="14">
-        <v>1.06205582454581</v>
-      </c>
-      <c r="I14" s="14">
-        <v>0.47739999999999999</v>
-      </c>
-      <c r="J14" s="14">
-        <v>0.11107551172966013</v>
-      </c>
-      <c r="K14" s="14">
-        <v>0</v>
-      </c>
-      <c r="L14" s="14">
-        <v>1.011691375024679</v>
-      </c>
-      <c r="M14" s="14">
-        <v>0.56205045247263075</v>
-      </c>
-      <c r="N14" s="21">
-        <v>1.4841131607226035</v>
-      </c>
-      <c r="O14" s="23">
-        <v>7.5445007460298559</v>
-      </c>
-      <c r="P14" s="23">
-        <v>9.1</v>
-      </c>
-      <c r="Q14" s="23">
-        <v>5.0414052649559933</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" s="14">
-        <v>2.4787267316625954</v>
-      </c>
-      <c r="E15" s="14">
-        <v>1.5072935699864518</v>
-      </c>
-      <c r="F15" s="14">
-        <v>0.13114731930321041</v>
-      </c>
-      <c r="G15" s="14">
-        <v>1.9058703261018888</v>
-      </c>
-      <c r="H15" s="14">
-        <v>0</v>
-      </c>
-      <c r="I15" s="14">
-        <v>0.41110000000000002</v>
-      </c>
-      <c r="J15" s="14">
-        <v>0</v>
-      </c>
-      <c r="K15" s="14">
-        <v>1.0368879452299757</v>
-      </c>
-      <c r="L15" s="14">
-        <v>0.89229699812925367</v>
-      </c>
-      <c r="M15" s="14">
-        <v>1.2604968981368243</v>
-      </c>
-      <c r="N15" s="21">
-        <v>0.43494800834006392</v>
-      </c>
-      <c r="O15" s="23">
-        <v>7.9562092224762884</v>
-      </c>
-      <c r="P15" s="23">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="Q15" s="23">
-        <v>7.2304756924160642</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="14">
-        <v>12.036462028653192</v>
-      </c>
-      <c r="E16" s="14">
-        <v>14.690826870034272</v>
-      </c>
-      <c r="F16" s="14">
-        <v>2.4571173079700253</v>
-      </c>
-      <c r="G16" s="14">
-        <v>4.8604171260649736</v>
-      </c>
-      <c r="H16" s="14">
-        <v>1.8174089333614543</v>
-      </c>
-      <c r="I16" s="14">
-        <v>2.0588000000000002</v>
-      </c>
-      <c r="J16" s="14">
-        <v>2.566584561254897</v>
-      </c>
-      <c r="K16" s="14">
-        <v>1.9537658797263695</v>
-      </c>
-      <c r="L16" s="14">
-        <v>2.1781909222789975</v>
-      </c>
-      <c r="M16" s="14">
-        <v>2.4816289901846873</v>
-      </c>
-      <c r="N16" s="21">
-        <v>4.5037215639801795</v>
-      </c>
-      <c r="O16" s="23">
-        <v>8.1696953402867685</v>
-      </c>
-      <c r="P16" s="23">
-        <v>6.7</v>
-      </c>
-      <c r="Q16" s="23">
-        <v>5.636136560567035</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="14">
-        <v>8.3331494569001308</v>
-      </c>
-      <c r="E17" s="14">
-        <v>3.6874208696079878</v>
-      </c>
-      <c r="F17" s="14">
-        <v>2.2967063175794622</v>
-      </c>
-      <c r="G17" s="14">
-        <v>4.0113695837012733</v>
-      </c>
-      <c r="H17" s="14">
-        <v>0.42340246664306652</v>
-      </c>
-      <c r="I17" s="14">
-        <v>1.1879</v>
-      </c>
-      <c r="J17" s="14">
-        <v>0.82824784717641098</v>
-      </c>
-      <c r="K17" s="14">
-        <v>0</v>
-      </c>
-      <c r="L17" s="14">
-        <v>0</v>
-      </c>
-      <c r="M17" s="14">
-        <v>0.88079865305212723</v>
-      </c>
-      <c r="N17" s="21">
-        <v>0</v>
-      </c>
-      <c r="O17" s="23">
-        <v>2.0701729813092102</v>
-      </c>
-      <c r="P17" s="23">
-        <v>0.5</v>
-      </c>
-      <c r="Q17" s="23">
-        <v>0.28220429532766028</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="14">
-        <v>5.0122940777216947</v>
-      </c>
-      <c r="E18" s="14">
-        <v>8.4390180594440558</v>
-      </c>
-      <c r="F18" s="14">
-        <v>0.9048113995307433</v>
-      </c>
-      <c r="G18" s="14">
-        <v>0</v>
-      </c>
-      <c r="H18" s="14">
-        <v>0</v>
-      </c>
-      <c r="I18" s="14">
-        <v>0</v>
-      </c>
-      <c r="J18" s="14">
-        <v>0</v>
-      </c>
-      <c r="K18" s="14">
-        <v>0</v>
-      </c>
-      <c r="L18" s="14">
-        <v>0</v>
-      </c>
-      <c r="M18" s="14">
-        <v>0</v>
-      </c>
-      <c r="N18" s="21">
-        <v>0</v>
-      </c>
-      <c r="O18" s="23">
-        <v>2.6482523478927704</v>
-      </c>
-      <c r="P18" s="23">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="Q18" s="23">
-        <v>4.1787877227366739</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="14">
-        <v>3.5353129806100583</v>
-      </c>
-      <c r="E19" s="14">
-        <v>4.8599509512033325</v>
-      </c>
-      <c r="F19" s="14">
-        <v>3.8945633266892905</v>
-      </c>
-      <c r="G19" s="14">
-        <v>2.0810969960991046</v>
-      </c>
-      <c r="H19" s="14">
-        <v>3.1927887343841532</v>
-      </c>
-      <c r="I19" s="14">
-        <v>1.6887000000000001</v>
-      </c>
-      <c r="J19" s="14">
-        <v>3.1263372864926211</v>
-      </c>
-      <c r="K19" s="14">
-        <v>1.6870705087645406</v>
-      </c>
-      <c r="L19" s="14">
-        <v>0.32414908639895251</v>
-      </c>
-      <c r="M19" s="14">
-        <v>0.16260204281171109</v>
-      </c>
-      <c r="N19" s="21">
-        <v>1.3481169038547842</v>
-      </c>
-      <c r="O19" s="23">
-        <v>3.9561647100749857</v>
-      </c>
-      <c r="P19" s="23">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="Q19" s="23">
-        <v>4.5216072733589767</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="14">
-        <v>0.53092532677015958</v>
-      </c>
-      <c r="E20" s="14">
-        <v>1.0193281509036862</v>
-      </c>
-      <c r="F20" s="14">
-        <v>1.1684706283465978</v>
-      </c>
-      <c r="G20" s="14">
-        <v>0.96005330035931602</v>
-      </c>
-      <c r="H20" s="14">
-        <v>0</v>
-      </c>
-      <c r="I20" s="14">
-        <v>0.78439999999999999</v>
-      </c>
-      <c r="J20" s="14">
-        <v>0</v>
-      </c>
-      <c r="K20" s="14">
-        <v>0</v>
-      </c>
-      <c r="L20" s="14">
-        <v>0.32812063618010201</v>
-      </c>
-      <c r="M20" s="14">
-        <v>0</v>
-      </c>
-      <c r="N20" s="21">
-        <v>0.28229127286371936</v>
-      </c>
-      <c r="O20" s="23">
-        <v>9.4645167179465837</v>
-      </c>
-      <c r="P20" s="23">
-        <v>3.9</v>
-      </c>
-      <c r="Q20" s="23">
-        <v>5.6913920534882436</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A21" s="10" t="s">
+    <row r="22" spans="1:18">
+      <c r="A22" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="16">
-        <v>3.5070632421313164</v>
-      </c>
-      <c r="H21" s="16">
-        <v>3.1020289567965551</v>
-      </c>
-      <c r="I21" s="16">
-        <v>1.7009000000000001</v>
-      </c>
-      <c r="J21" s="16">
-        <v>0</v>
-      </c>
-      <c r="K21" s="16">
-        <v>1.1812990540391501</v>
-      </c>
-      <c r="L21" s="16">
-        <v>0.55610781362635098</v>
-      </c>
-      <c r="M21" s="16">
-        <v>0</v>
-      </c>
-      <c r="N21" s="22">
-        <v>0</v>
-      </c>
-      <c r="O21" s="24">
-        <v>3.1019579996103404</v>
-      </c>
-      <c r="P21" s="24">
-        <v>7</v>
-      </c>
-      <c r="Q21" s="24">
-        <v>1.3988584602956362</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" s="9" customFormat="1">
-      <c r="A22" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>19</v>
+      <c r="C22" s="24" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>